<commit_message>
feat: setup colab on IDE
</commit_message>
<xml_diff>
--- a/data/List_Cafe_Model_Final.xlsx
+++ b/data/List_Cafe_Model_Final.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S99"/>
+  <dimension ref="A1:S111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6032,7 +6032,11 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="S86" t="inlineStr"/>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Sangat Dekat</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6874,6 +6878,786 @@
         </is>
       </c>
       <c r="S99" t="inlineStr">
+        <is>
+          <t>Jauh</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Ulansa Coffee</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C100" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="D100" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E100" t="n">
+        <v>8</v>
+      </c>
+      <c r="F100" t="n">
+        <v>4</v>
+      </c>
+      <c r="G100" t="n">
+        <v>15</v>
+      </c>
+      <c r="H100" t="n">
+        <v>1</v>
+      </c>
+      <c r="I100" t="n">
+        <v>1</v>
+      </c>
+      <c r="J100" t="n">
+        <v>1</v>
+      </c>
+      <c r="K100" t="n">
+        <v>1</v>
+      </c>
+      <c r="L100" t="n">
+        <v>1</v>
+      </c>
+      <c r="M100" t="n">
+        <v>1</v>
+      </c>
+      <c r="N100" t="n">
+        <v>1</v>
+      </c>
+      <c r="O100" t="n">
+        <v>1</v>
+      </c>
+      <c r="P100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Janimani</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C101" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D101" t="n">
+        <v>13</v>
+      </c>
+      <c r="E101" t="n">
+        <v>8</v>
+      </c>
+      <c r="F101" t="n">
+        <v>4</v>
+      </c>
+      <c r="G101" t="n">
+        <v>14</v>
+      </c>
+      <c r="H101" t="n">
+        <v>1</v>
+      </c>
+      <c r="I101" t="n">
+        <v>1</v>
+      </c>
+      <c r="J101" t="n">
+        <v>1</v>
+      </c>
+      <c r="K101" t="n">
+        <v>1</v>
+      </c>
+      <c r="L101" t="n">
+        <v>1</v>
+      </c>
+      <c r="M101" t="n">
+        <v>1</v>
+      </c>
+      <c r="N101" t="n">
+        <v>1</v>
+      </c>
+      <c r="O101" t="n">
+        <v>1</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0</v>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Jauh</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Toko Kopi Jaya Ijen</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C102" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D102" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E102" t="n">
+        <v>8</v>
+      </c>
+      <c r="F102" t="n">
+        <v>4</v>
+      </c>
+      <c r="G102" t="n">
+        <v>15</v>
+      </c>
+      <c r="H102" t="n">
+        <v>1</v>
+      </c>
+      <c r="I102" t="n">
+        <v>1</v>
+      </c>
+      <c r="J102" t="n">
+        <v>1</v>
+      </c>
+      <c r="K102" t="n">
+        <v>1</v>
+      </c>
+      <c r="L102" t="n">
+        <v>1</v>
+      </c>
+      <c r="M102" t="n">
+        <v>1</v>
+      </c>
+      <c r="N102" t="n">
+        <v>1</v>
+      </c>
+      <c r="O102" t="n">
+        <v>1</v>
+      </c>
+      <c r="P102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Jauh</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Toko Kopi Jaya Kepundung</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C103" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D103" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E103" t="n">
+        <v>8</v>
+      </c>
+      <c r="F103" t="n">
+        <v>4</v>
+      </c>
+      <c r="G103" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H103" t="n">
+        <v>1</v>
+      </c>
+      <c r="I103" t="n">
+        <v>1</v>
+      </c>
+      <c r="J103" t="n">
+        <v>1</v>
+      </c>
+      <c r="K103" t="n">
+        <v>1</v>
+      </c>
+      <c r="L103" t="n">
+        <v>1</v>
+      </c>
+      <c r="M103" t="n">
+        <v>1</v>
+      </c>
+      <c r="N103" t="n">
+        <v>1</v>
+      </c>
+      <c r="O103" t="n">
+        <v>1</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0</v>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Jauh</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Toko Kopi Jaya FEB UB</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>5</v>
+      </c>
+      <c r="C104" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D104" t="n">
+        <v>13</v>
+      </c>
+      <c r="E104" t="n">
+        <v>8</v>
+      </c>
+      <c r="F104" t="n">
+        <v>4</v>
+      </c>
+      <c r="G104" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H104" t="n">
+        <v>1</v>
+      </c>
+      <c r="I104" t="n">
+        <v>1</v>
+      </c>
+      <c r="J104" t="n">
+        <v>1</v>
+      </c>
+      <c r="K104" t="n">
+        <v>1</v>
+      </c>
+      <c r="L104" t="n">
+        <v>1</v>
+      </c>
+      <c r="M104" t="n">
+        <v>1</v>
+      </c>
+      <c r="N104" t="n">
+        <v>1</v>
+      </c>
+      <c r="O104" t="n">
+        <v>1</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0</v>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Toko Kopi Jaya Klojen</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C105" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="D105" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E105" t="n">
+        <v>8</v>
+      </c>
+      <c r="F105" t="n">
+        <v>4</v>
+      </c>
+      <c r="G105" t="n">
+        <v>15</v>
+      </c>
+      <c r="H105" t="n">
+        <v>1</v>
+      </c>
+      <c r="I105" t="n">
+        <v>1</v>
+      </c>
+      <c r="J105" t="n">
+        <v>1</v>
+      </c>
+      <c r="K105" t="n">
+        <v>1</v>
+      </c>
+      <c r="L105" t="n">
+        <v>1</v>
+      </c>
+      <c r="M105" t="n">
+        <v>1</v>
+      </c>
+      <c r="N105" t="n">
+        <v>1</v>
+      </c>
+      <c r="O105" t="n">
+        <v>1</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0</v>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>Jauh</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Toko Kopi Jaya Begawan</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C106" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D106" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E106" t="n">
+        <v>8</v>
+      </c>
+      <c r="F106" t="n">
+        <v>4</v>
+      </c>
+      <c r="G106" t="n">
+        <v>14</v>
+      </c>
+      <c r="H106" t="n">
+        <v>1</v>
+      </c>
+      <c r="I106" t="n">
+        <v>1</v>
+      </c>
+      <c r="J106" t="n">
+        <v>1</v>
+      </c>
+      <c r="K106" t="n">
+        <v>1</v>
+      </c>
+      <c r="L106" t="n">
+        <v>1</v>
+      </c>
+      <c r="M106" t="n">
+        <v>1</v>
+      </c>
+      <c r="N106" t="n">
+        <v>1</v>
+      </c>
+      <c r="O106" t="n">
+        <v>1</v>
+      </c>
+      <c r="P106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>Dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Toko Kopi Jaya Suhat</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="C107" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D107" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E107" t="n">
+        <v>8</v>
+      </c>
+      <c r="F107" t="n">
+        <v>4</v>
+      </c>
+      <c r="G107" t="n">
+        <v>24</v>
+      </c>
+      <c r="H107" t="n">
+        <v>1</v>
+      </c>
+      <c r="I107" t="n">
+        <v>1</v>
+      </c>
+      <c r="J107" t="n">
+        <v>1</v>
+      </c>
+      <c r="K107" t="n">
+        <v>1</v>
+      </c>
+      <c r="L107" t="n">
+        <v>1</v>
+      </c>
+      <c r="M107" t="n">
+        <v>1</v>
+      </c>
+      <c r="N107" t="n">
+        <v>1</v>
+      </c>
+      <c r="O107" t="n">
+        <v>1</v>
+      </c>
+      <c r="P107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Halter Coffee</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C108" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D108" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="E108" t="n">
+        <v>8</v>
+      </c>
+      <c r="F108" t="n">
+        <v>4</v>
+      </c>
+      <c r="G108" t="n">
+        <v>13</v>
+      </c>
+      <c r="H108" t="n">
+        <v>1</v>
+      </c>
+      <c r="I108" t="n">
+        <v>1</v>
+      </c>
+      <c r="J108" t="n">
+        <v>1</v>
+      </c>
+      <c r="K108" t="n">
+        <v>1</v>
+      </c>
+      <c r="L108" t="n">
+        <v>1</v>
+      </c>
+      <c r="M108" t="n">
+        <v>1</v>
+      </c>
+      <c r="N108" t="n">
+        <v>1</v>
+      </c>
+      <c r="O108" t="n">
+        <v>1</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Jauh</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Lupa Lelah Cafe</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D109" t="n">
+        <v>13</v>
+      </c>
+      <c r="E109" t="n">
+        <v>8</v>
+      </c>
+      <c r="F109" t="n">
+        <v>4</v>
+      </c>
+      <c r="G109" t="n">
+        <v>24</v>
+      </c>
+      <c r="H109" t="n">
+        <v>1</v>
+      </c>
+      <c r="I109" t="n">
+        <v>1</v>
+      </c>
+      <c r="J109" t="n">
+        <v>1</v>
+      </c>
+      <c r="K109" t="n">
+        <v>1</v>
+      </c>
+      <c r="L109" t="n">
+        <v>1</v>
+      </c>
+      <c r="M109" t="n">
+        <v>1</v>
+      </c>
+      <c r="N109" t="n">
+        <v>1</v>
+      </c>
+      <c r="O109" t="n">
+        <v>1</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Begati Coffee</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C110" t="n">
+        <v>2</v>
+      </c>
+      <c r="D110" t="n">
+        <v>13</v>
+      </c>
+      <c r="E110" t="n">
+        <v>7</v>
+      </c>
+      <c r="F110" t="n">
+        <v>4</v>
+      </c>
+      <c r="G110" t="n">
+        <v>24</v>
+      </c>
+      <c r="H110" t="n">
+        <v>1</v>
+      </c>
+      <c r="I110" t="n">
+        <v>1</v>
+      </c>
+      <c r="J110" t="n">
+        <v>1</v>
+      </c>
+      <c r="K110" t="n">
+        <v>1</v>
+      </c>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" t="n">
+        <v>1</v>
+      </c>
+      <c r="N110" t="n">
+        <v>1</v>
+      </c>
+      <c r="O110" t="n">
+        <v>1</v>
+      </c>
+      <c r="P110" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Equal Coffee Roastery</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C111" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D111" t="n">
+        <v>13</v>
+      </c>
+      <c r="E111" t="n">
+        <v>8</v>
+      </c>
+      <c r="F111" t="n">
+        <v>4</v>
+      </c>
+      <c r="G111" t="n">
+        <v>16</v>
+      </c>
+      <c r="H111" t="n">
+        <v>1</v>
+      </c>
+      <c r="I111" t="n">
+        <v>1</v>
+      </c>
+      <c r="J111" t="n">
+        <v>1</v>
+      </c>
+      <c r="K111" t="n">
+        <v>1</v>
+      </c>
+      <c r="L111" t="n">
+        <v>1</v>
+      </c>
+      <c r="M111" t="n">
+        <v>1</v>
+      </c>
+      <c r="N111" t="n">
+        <v>1</v>
+      </c>
+      <c r="O111" t="n">
+        <v>1</v>
+      </c>
+      <c r="P111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
         <is>
           <t>Jauh</t>
         </is>

</xml_diff>